<commit_message>
Update Intäkt Budget for Grimmered
</commit_message>
<xml_diff>
--- a/data/Grimmered/Intäkt Budget VC (37).xlsx
+++ b/data/Grimmered/Intäkt Budget VC (37).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ezzat.rajab.AD\claude-workspace\VGR Alla enheter\103\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ezzat.rajab.AD\claude-workspace\VGR Alla enheter\Dashboard\data\Grimmered\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80839EDF-FCA1-4FB7-91F4-CA5EC0E671A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB6145A8-8BA4-4D81-AFC9-6A8006659B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -94,7 +94,7 @@
     <t>Tillämpade filter:
 Category är VCRevenueModule
 Value är SEK
-Inkluderade (1) VC VGR (Cost Center Type) + VC StorGöteborg (Business Area) + 102 Frölunda Torg (Name)
+Inkluderade (1) VC VGR (Cost Center Type) + VC StorGöteborg (Business Area) + 103 Grimmered (Name)
 Year är 2026</t>
   </si>
 </sst>
@@ -623,40 +623,40 @@
         <v>16</v>
       </c>
       <c r="B4" s="5">
-        <v>0.32743899999999998</v>
+        <v>0.31560300000000002</v>
       </c>
       <c r="C4" s="5">
-        <v>0.32846700000000001</v>
+        <v>0.31612400000000002</v>
       </c>
       <c r="D4" s="5">
-        <v>0.32888299999999998</v>
+        <v>0.31664300000000001</v>
       </c>
       <c r="E4" s="5">
-        <v>0.32929799999999998</v>
+        <v>0.31715900000000002</v>
       </c>
       <c r="F4" s="5">
-        <v>0.32971</v>
+        <v>0.31767200000000001</v>
       </c>
       <c r="G4" s="5">
-        <v>0.33012000000000002</v>
+        <v>0.31818200000000002</v>
       </c>
       <c r="H4" s="5">
-        <v>0.33052900000000002</v>
+        <v>0.318689</v>
       </c>
       <c r="I4" s="5">
-        <v>0.32973599999999997</v>
+        <v>0.317803</v>
       </c>
       <c r="J4" s="5">
-        <v>0.33014399999999999</v>
+        <v>0.31786700000000001</v>
       </c>
       <c r="K4" s="5">
-        <v>0.33054899999999998</v>
+        <v>0.31814999999999999</v>
       </c>
       <c r="L4" s="5">
-        <v>0.33095200000000002</v>
+        <v>0.31843199999999999</v>
       </c>
       <c r="M4" s="5">
-        <v>0.33135399999999998</v>
+        <v>0.31849300000000003</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -664,40 +664,40 @@
         <v>17</v>
       </c>
       <c r="B5" s="4">
-        <v>1425735</v>
+        <v>1181475</v>
       </c>
       <c r="C5" s="4">
-        <v>1433700</v>
+        <v>1186785</v>
       </c>
       <c r="D5" s="4">
-        <v>1439010</v>
+        <v>1192095</v>
       </c>
       <c r="E5" s="4">
-        <v>1444320</v>
+        <v>1197405</v>
       </c>
       <c r="F5" s="4">
-        <v>1449630</v>
+        <v>1202715</v>
       </c>
       <c r="G5" s="4">
-        <v>1454940</v>
+        <v>1208025</v>
       </c>
       <c r="H5" s="4">
-        <v>1460250</v>
+        <v>1213335</v>
       </c>
       <c r="I5" s="4">
-        <v>1460250</v>
+        <v>1213335</v>
       </c>
       <c r="J5" s="4">
-        <v>1465560</v>
+        <v>1218645</v>
       </c>
       <c r="K5" s="4">
-        <v>1470870</v>
+        <v>1223955</v>
       </c>
       <c r="L5" s="4">
-        <v>1476180</v>
+        <v>1229265</v>
       </c>
       <c r="M5" s="4">
-        <v>1481490</v>
+        <v>1234575</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -705,40 +705,40 @@
         <v>18</v>
       </c>
       <c r="B6" s="4">
-        <v>2711.85</v>
+        <v>2047</v>
       </c>
       <c r="C6" s="4">
-        <v>2727</v>
+        <v>2056.1999999999998</v>
       </c>
       <c r="D6" s="4">
-        <v>2737.1</v>
+        <v>2065.4</v>
       </c>
       <c r="E6" s="4">
-        <v>2774.4</v>
+        <v>2097.15</v>
       </c>
       <c r="F6" s="4">
-        <v>2784.6</v>
+        <v>2106.4499999999998</v>
       </c>
       <c r="G6" s="4">
-        <v>2794.8</v>
+        <v>2115.75</v>
       </c>
       <c r="H6" s="4">
-        <v>2805</v>
+        <v>2125.0500000000002</v>
       </c>
       <c r="I6" s="4">
-        <v>2805</v>
+        <v>2125.0500000000002</v>
       </c>
       <c r="J6" s="4">
-        <v>2842.8</v>
+        <v>2157.3000000000002</v>
       </c>
       <c r="K6" s="4">
-        <v>2853.1</v>
+        <v>2166.6999999999998</v>
       </c>
       <c r="L6" s="4">
-        <v>2863.4</v>
+        <v>2176.1</v>
       </c>
       <c r="M6" s="4">
-        <v>2873.7</v>
+        <v>2185.5</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -746,40 +746,40 @@
         <v>19</v>
       </c>
       <c r="B7" s="4">
-        <v>1439992.35</v>
+        <v>1086957</v>
       </c>
       <c r="C7" s="4">
-        <v>1448037</v>
+        <v>1091842.2</v>
       </c>
       <c r="D7" s="4">
-        <v>1453400.1</v>
+        <v>1096727.3999999999</v>
       </c>
       <c r="E7" s="4">
-        <v>1473206.4</v>
+        <v>1113586.6499999999</v>
       </c>
       <c r="F7" s="4">
-        <v>1478622.6</v>
+        <v>1118524.95</v>
       </c>
       <c r="G7" s="4">
-        <v>1484038.8</v>
+        <v>1123463.25</v>
       </c>
       <c r="H7" s="4">
-        <v>1489455</v>
+        <v>1128401.55</v>
       </c>
       <c r="I7" s="4">
-        <v>1489455</v>
+        <v>1128401.55</v>
       </c>
       <c r="J7" s="4">
-        <v>1509526.8</v>
+        <v>1145526.3</v>
       </c>
       <c r="K7" s="4">
-        <v>1514996.1</v>
+        <v>1150517.7</v>
       </c>
       <c r="L7" s="4">
-        <v>1520465.4</v>
+        <v>1155509.1000000001</v>
       </c>
       <c r="M7" s="4">
-        <v>1525934.7</v>
+        <v>1160500.5</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -787,40 +787,40 @@
         <v>20</v>
       </c>
       <c r="B8" s="4">
-        <v>1.01</v>
+        <v>0.92</v>
       </c>
       <c r="C8" s="4">
-        <v>1.01</v>
+        <v>0.92</v>
       </c>
       <c r="D8" s="4">
-        <v>1.01</v>
+        <v>0.92</v>
       </c>
       <c r="E8" s="4">
-        <v>1.02</v>
+        <v>0.93</v>
       </c>
       <c r="F8" s="4">
-        <v>1.02</v>
+        <v>0.93</v>
       </c>
       <c r="G8" s="4">
-        <v>1.02</v>
+        <v>0.93</v>
       </c>
       <c r="H8" s="4">
-        <v>1.02</v>
+        <v>0.93</v>
       </c>
       <c r="I8" s="4">
-        <v>1.02</v>
+        <v>0.93</v>
       </c>
       <c r="J8" s="4">
-        <v>1.03</v>
+        <v>0.94</v>
       </c>
       <c r="K8" s="4">
-        <v>1.03</v>
+        <v>0.94</v>
       </c>
       <c r="L8" s="4">
-        <v>1.03</v>
+        <v>0.94</v>
       </c>
       <c r="M8" s="4">
-        <v>1.03</v>
+        <v>0.94</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -828,40 +828,40 @@
         <v>21</v>
       </c>
       <c r="B9" s="4">
-        <v>8200</v>
+        <v>7050</v>
       </c>
       <c r="C9" s="4">
-        <v>8220</v>
+        <v>7070</v>
       </c>
       <c r="D9" s="4">
-        <v>8240</v>
+        <v>7090</v>
       </c>
       <c r="E9" s="4">
-        <v>8260</v>
+        <v>7110</v>
       </c>
       <c r="F9" s="4">
-        <v>8280</v>
+        <v>7130</v>
       </c>
       <c r="G9" s="4">
-        <v>8300</v>
+        <v>7150</v>
       </c>
       <c r="H9" s="4">
-        <v>8320</v>
+        <v>7170</v>
       </c>
       <c r="I9" s="4">
-        <v>8340</v>
+        <v>7190</v>
       </c>
       <c r="J9" s="4">
-        <v>8360</v>
+        <v>7220</v>
       </c>
       <c r="K9" s="4">
-        <v>8380</v>
+        <v>7245</v>
       </c>
       <c r="L9" s="4">
-        <v>8400</v>
+        <v>7270</v>
       </c>
       <c r="M9" s="4">
-        <v>8420</v>
+        <v>7300</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -869,40 +869,40 @@
         <v>22</v>
       </c>
       <c r="B10" s="4">
-        <v>2685</v>
+        <v>2225</v>
       </c>
       <c r="C10" s="4">
-        <v>2700</v>
+        <v>2235</v>
       </c>
       <c r="D10" s="4">
-        <v>2710</v>
+        <v>2245</v>
       </c>
       <c r="E10" s="4">
-        <v>2720</v>
+        <v>2255</v>
       </c>
       <c r="F10" s="4">
-        <v>2730</v>
+        <v>2265</v>
       </c>
       <c r="G10" s="4">
-        <v>2740</v>
+        <v>2275</v>
       </c>
       <c r="H10" s="4">
-        <v>2750</v>
+        <v>2285</v>
       </c>
       <c r="I10" s="4">
-        <v>2750</v>
+        <v>2285</v>
       </c>
       <c r="J10" s="4">
-        <v>2760</v>
+        <v>2295</v>
       </c>
       <c r="K10" s="4">
-        <v>2770</v>
+        <v>2305</v>
       </c>
       <c r="L10" s="4">
-        <v>2780</v>
+        <v>2315</v>
       </c>
       <c r="M10" s="4">
-        <v>2790</v>
+        <v>2325</v>
       </c>
     </row>
     <row r="12" spans="1:13">

</xml_diff>